<commit_message>
fix: redesign skip_rows test to match actual behavior (skips after header)
</commit_message>
<xml_diff>
--- a/demos/excel/excel-options-testbench/data/03_skip_rows.xlsx
+++ b/demos/excel/excel-options-testbench/data/03_skip_rows.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,75 +419,108 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Generated: 2024-06-15</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>project</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Department: Engineering</t>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Confidential — Internal Use Only</t>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bravo</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>85</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>project</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
+          <t>Charlie</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alpha</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Planning</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Echo</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>85</v>
+        <v>160</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -497,15 +530,15 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Charlie</t>
+          <t>Foxtrot</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -515,15 +548,15 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Golf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>45</v>
+        <v>210</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -533,15 +566,15 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Echo</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>160</v>
+        <v>75</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>

</xml_diff>